<commit_message>
change jpg to webp
</commit_message>
<xml_diff>
--- a/data/DATA.xlsx
+++ b/data/DATA.xlsx
@@ -2186,7 +2186,7 @@
     <t>Mặt hơi nhiều râu</t>
   </si>
   <si>
-    <t>./images/2012/TRUONG_MINH_Y.jpg</t>
+    <t>./images/2012/TRUONG_MINH_Y.webp</t>
   </si>
   <si>
     <t>Định Hưng (Toni)</t>
@@ -2198,7 +2198,7 @@
     <t>Toni Định</t>
   </si>
   <si>
-    <t>./images/2012/DINH_HUNG.jpg</t>
+    <t>./images/2012/DINH_HUNG.webp</t>
   </si>
   <si>
     <t>Trương Thị Phương Anh (Bơ Cena)</t>
@@ -2207,7 +2207,7 @@
     <t>Chị Bơ</t>
   </si>
   <si>
-    <t>./images/2012/TRUONG_THI_PHUONG_ANH.jpg</t>
+    <t>./images/2012/TRUONG_THI_PHUONG_ANH.webp</t>
   </si>
   <si>
     <t>Lê Thị Bích Tiên</t>
@@ -2216,7 +2216,7 @@
     <t>Giọng to nhất Chánh Tâm</t>
   </si>
   <si>
-    <t>./images/2012/LE_THI_BICH_TIEN.jpg</t>
+    <t>./images/2012/LE_THI_BICH_TIEN.webp</t>
   </si>
   <si>
     <t>Tống Văn Hùng</t>
@@ -2225,7 +2225,7 @@
     <t>Hùng hóm hỉnh</t>
   </si>
   <si>
-    <t>./images/2011/TONG_VAN_HUNG.jpg</t>
+    <t>./images/2011/TONG_VAN_HUNG.webp</t>
   </si>
   <si>
     <t>Trương Thị Kim Chi (Xuxuchichi)</t>
@@ -2237,7 +2237,7 @@
     <t>Cô dâu Chi</t>
   </si>
   <si>
-    <t>./images/2011/TRUONG_THI_KIM_CHI.jpg</t>
+    <t>./images/2011/TRUONG_THI_KIM_CHI.webp</t>
   </si>
   <si>
     <t>Trương Thị Kim Cương</t>
@@ -2246,7 +2246,7 @@
     <t>Mẹ Khoai, Đậu, Dâu Tây</t>
   </si>
   <si>
-    <t>./images/2011/TRUONG_THI_KIM_CUONG.jpg</t>
+    <t>./images/2011/TRUONG_THI_KIM_CUONG.webp</t>
   </si>
   <si>
     <t>Hồ Thị Diệu Thảo (Bông)</t>
@@ -2255,7 +2255,7 @@
     <t>Tâm Thuận</t>
   </si>
   <si>
-    <t>./images/2011/HO_THI_DIEU_THAO.jpg</t>
+    <t>./images/2011/HO_THI_DIEU_THAO.webp</t>
   </si>
   <si>
     <t>Phan Thị Thanh Hồng</t>
@@ -2264,7 +2264,7 @@
     <t>Quảng Tuyết</t>
   </si>
   <si>
-    <t>./images/2011/PHAN_THI_THANH_HONG.jpg</t>
+    <t>./images/2011/PHAN_THI_THANH_HONG.webp</t>
   </si>
   <si>
     <t>full_name 2010</t>
@@ -9601,8 +9601,8 @@
       <c r="C2" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
+      <c r="D2" s="2" t="s">
+        <v>686</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>711</v>
@@ -9610,7 +9610,7 @@
       <c r="F2" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>713</v>
       </c>
       <c r="H2" s="2">
@@ -9636,7 +9636,7 @@
       <c r="F3" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>717</v>
       </c>
       <c r="H3" s="2">
@@ -9688,7 +9688,7 @@
       <c r="F5" s="1" t="s">
         <v>722</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>723</v>
       </c>
       <c r="H5" s="2">
@@ -10757,7 +10757,7 @@
       <c r="F2" s="1" t="s">
         <v>725</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>726</v>
       </c>
       <c r="H2" s="2">
@@ -10783,7 +10783,7 @@
       <c r="F3" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>730</v>
       </c>
       <c r="H3" s="2">
@@ -10809,7 +10809,7 @@
       <c r="F4" s="1" t="s">
         <v>732</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>733</v>
       </c>
       <c r="H4" s="2">
@@ -10835,7 +10835,7 @@
       <c r="F5" s="1" t="s">
         <v>735</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>736</v>
       </c>
       <c r="H5" s="1">
@@ -10861,7 +10861,7 @@
       <c r="F6" s="1" t="s">
         <v>738</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="2" t="s">
         <v>739</v>
       </c>
       <c r="H6" s="2">

</xml_diff>

<commit_message>
change jpg to webp (2018~2020)
</commit_message>
<xml_diff>
--- a/data/DATA.xlsx
+++ b/data/DATA.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1891" uniqueCount="851">
   <si>
     <t>id</t>
   </si>
@@ -1810,7 +1810,7 @@
     <t>Nhật Uyên xinh đẹp</t>
   </si>
   <si>
-    <t>./data/images/2020/NGUYEN_NHAT_UYEN.jpg</t>
+    <t>./data/images/2020/NGUYEN_NHAT_UYEN.webp</t>
   </si>
   <si>
     <t>Nguyễn Nhật Linh</t>
@@ -1819,7 +1819,7 @@
     <t>Bớt nghe, bớt nói, bớt nhìn. Giữ tâm thanh tịnh mới là thảnh thơi.</t>
   </si>
   <si>
-    <t>./data/images/2020/NGUYEN_NHAT_LINH.jpg</t>
+    <t>./data/images/2020/NGUYEN_NHAT_LINH.webp</t>
   </si>
   <si>
     <t>Trần Xuân Trung</t>
@@ -1828,13 +1828,16 @@
     <t>Trung</t>
   </si>
   <si>
+    <t>./data/images/2020/TRAN_XUAN_TRUNG.webp</t>
+  </si>
+  <si>
     <t>Nguyễn Thị Mỹ Nhàn</t>
   </si>
   <si>
     <t>Nhuận Niệm</t>
   </si>
   <si>
-    <t>./data/images/2020/NGUYEN_THI_MY_NHAN.jpg</t>
+    <t>./data/images/2020/NGUYEN_THI_MY_NHAN.webp</t>
   </si>
   <si>
     <t>Nguyễn Đăng Huy</t>
@@ -1843,7 +1846,7 @@
     <t>Chú Huy</t>
   </si>
   <si>
-    <t>./data/images/2020/NGUYEN_DANG_HUY.jpg</t>
+    <t>./data/images/2020/NGUYEN_DANG_HUY.webp</t>
   </si>
   <si>
     <t>Hoàng Giang (Long Ka)</t>
@@ -1852,7 +1855,7 @@
     <t>Kết nối - Nhiệt tình - Vui vẻ - Hoà đồng</t>
   </si>
   <si>
-    <t>./data/images/2020/HOANG_GIANG.jpg</t>
+    <t>./data/images/2020/HOANG_GIANG.webp</t>
   </si>
   <si>
     <t>Nguyễn Bá Quốc</t>
@@ -1864,6 +1867,9 @@
     <t>Phan Văn Hưng</t>
   </si>
   <si>
+    <t>./data/images/2020/PHAN_VAN_HUNG.webp</t>
+  </si>
+  <si>
     <t>Nguyễn Phúc Hưng (Ki)</t>
   </si>
   <si>
@@ -1873,7 +1879,7 @@
     <t>Banh</t>
   </si>
   <si>
-    <t>./data/images/2020/DINH_THI_NGOC_ANH.jpg</t>
+    <t>./data/images/2020/DINH_THI_NGOC_ANH.webp</t>
   </si>
   <si>
     <t>Nguyễn Hoàng Kiều Anh</t>
@@ -1882,7 +1888,7 @@
     <t>Quang Tú</t>
   </si>
   <si>
-    <t>./data/images/2020/NGUYEN_HOANG_KIEU_ANH.jpg</t>
+    <t>./data/images/2020/NGUYEN_HOANG_KIEU_ANH.webp</t>
   </si>
   <si>
     <t>Đoàn Thị Thu Hà</t>
@@ -1891,7 +1897,7 @@
     <t>Cô gái Huế hay cười</t>
   </si>
   <si>
-    <t>./data/images/2020/DOAN_THI_THU_HA.jpg</t>
+    <t>./data/images/2020/DOAN_THI_THU_HA.webp</t>
   </si>
   <si>
     <t>Lê Thị Thuận Hóa</t>
@@ -1906,7 +1912,7 @@
     <t>Nàng thơ cây cỏ</t>
   </si>
   <si>
-    <t>./data/images/2019/LE_THI_THUAN_HOA.jpg</t>
+    <t>./data/images/2019/LE_THI_THUAN_HOA.webp</t>
   </si>
   <si>
     <t>Nguyễn Thị Như Ngọc</t>
@@ -1918,7 +1924,7 @@
     <t>Quảng Lan</t>
   </si>
   <si>
-    <t>./data/images/2019/NGUYEN_THI_NHU_NGOC.jpg</t>
+    <t>./data/images/2019/NGUYEN_THI_NHU_NGOC.webp</t>
   </si>
   <si>
     <t>Ngô Thị Bảo Trân</t>
@@ -1930,6 +1936,9 @@
     <t>Cô gái lúm đồng tiền 🪙</t>
   </si>
   <si>
+    <t>./data/images/2019/NGO_THI_BAO_TRAN.webp</t>
+  </si>
+  <si>
     <t>Ngô Đức Minh Tuệ</t>
   </si>
   <si>
@@ -1942,7 +1951,7 @@
     <t>Quảng Tịnh</t>
   </si>
   <si>
-    <t>./data/images/2019/NGUYEN_THI_THANH_HIEN.jpg</t>
+    <t>./data/images/2019/NGUYEN_THI_THANH_HIEN.webp</t>
   </si>
   <si>
     <t>Nguyễn Kính Nghĩa (Bin)</t>
@@ -1951,7 +1960,7 @@
     <t>Quảng Trung</t>
   </si>
   <si>
-    <t>./data/images/2019/NGUYEN_KINH_NGHIA.jpg</t>
+    <t>./data/images/2019/NGUYEN_KINH_NGHIA.webp</t>
   </si>
   <si>
     <t>Lê Đình Hùng</t>
@@ -1966,6 +1975,9 @@
     <t>Nhuận Tâm</t>
   </si>
   <si>
+    <t>./data/images/2019/LE_DINH_HUNG.webp</t>
+  </si>
+  <si>
     <t>Phan Vũ Phúc Dương (Hím em)</t>
   </si>
   <si>
@@ -1975,7 +1987,7 @@
     <t>vuýp</t>
   </si>
   <si>
-    <t>./data/images/2018/PHAN_VU_PHUC_DUONG.jpg</t>
+    <t>./data/images/2018/PHAN_VU_PHUC_DUONG.webp</t>
   </si>
   <si>
     <t>Nguyễn Thị Xuân Mai</t>
@@ -1987,7 +1999,7 @@
     <t>Quảng Trang</t>
   </si>
   <si>
-    <t>./data/images/2018/NGUYEN_THI_XUAN_MAI.jpg</t>
+    <t>./data/images/2018/NGUYEN_THI_XUAN_MAI.webp</t>
   </si>
   <si>
     <t>Lê Văn Anh Hào</t>
@@ -2002,7 +2014,7 @@
     <t>Quảng Châu</t>
   </si>
   <si>
-    <t>./data/images/2018/NGUYEN_LE_HONG_NGOC.jpg</t>
+    <t>./data/images/2018/NGUYEN_LE_HONG_NGOC.webp</t>
   </si>
   <si>
     <t>Nguyễn Thị Thanh Phương (Bơ nhỏ)</t>
@@ -2011,7 +2023,7 @@
     <t>Quảng Mỹ</t>
   </si>
   <si>
-    <t>./data/images/2018/NGUYEN_THI_THANH_PHUONG.jpg</t>
+    <t>./data/images/2018/NGUYEN_THI_THANH_PHUONG.webp</t>
   </si>
   <si>
     <t>Ngô Thị Băng Châu (Bắp)</t>
@@ -2020,7 +2032,7 @@
     <t>Nhuận Thảo</t>
   </si>
   <si>
-    <t>./data/images/2018/NGO_THI_BANG_CHAU.jpg</t>
+    <t>./data/images/2018/NGO_THI_BANG_CHAU.webp</t>
   </si>
   <si>
     <t>Lê Đức Duy</t>
@@ -4034,10 +4046,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>10</v>
@@ -4046,10 +4058,10 @@
         <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="H2" s="1">
         <v>5.0</v>
@@ -4060,22 +4072,22 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>585</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="H3" s="1">
         <v>3.0</v>
@@ -4086,7 +4098,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>360</v>
@@ -4098,10 +4110,10 @@
         <v>26</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="H4" s="1">
         <v>5.0</v>
@@ -4112,22 +4124,22 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>144</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="H5" s="1">
         <v>3.0</v>
@@ -4138,22 +4150,22 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>280</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="H6" s="1">
         <v>6.0</v>
@@ -4164,10 +4176,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>10</v>
@@ -4176,10 +4188,10 @@
         <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="H7" s="1">
         <v>6.0</v>
@@ -4190,22 +4202,22 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>139</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="H8" s="2">
         <v>7.0</v>
@@ -4216,22 +4228,22 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>39</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="H9" s="2">
         <v>7.0</v>
@@ -5281,22 +5293,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="H2" s="1">
         <v>5.0</v>
@@ -6351,22 +6363,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>532</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="H2" s="1">
         <v>5.0</v>
@@ -6377,10 +6389,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -6389,10 +6401,10 @@
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="H3" s="2">
         <v>6.0</v>
@@ -7446,22 +7458,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>377</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>52</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="H2" s="7">
         <v>5.0</v>
@@ -8516,10 +8528,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>10</v>
@@ -8528,7 +8540,7 @@
         <v>501</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="H2" s="2">
         <v>7.0</v>
@@ -8539,10 +8551,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>10</v>
@@ -9608,22 +9620,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>146</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="H2" s="2">
         <v>5.0</v>
@@ -9634,22 +9646,22 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>267</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="H3" s="2">
         <v>5.0</v>
@@ -9660,7 +9672,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>62</v>
@@ -9672,10 +9684,10 @@
         <v>52</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="H4" s="2">
         <v>5.0</v>
@@ -9686,22 +9698,22 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>175</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="H5" s="2">
         <v>5.0</v>
@@ -10755,22 +10767,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="H2" s="2">
         <v>6.0</v>
@@ -10781,22 +10793,22 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="H3" s="2">
         <v>5.0</v>
@@ -10807,22 +10819,22 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>441</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="H4" s="2">
         <v>5.0</v>
@@ -10833,7 +10845,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>71</v>
@@ -10845,10 +10857,10 @@
         <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="H5" s="1">
         <v>6.0</v>
@@ -10859,7 +10871,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>222</v>
@@ -10871,10 +10883,10 @@
         <v>11</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="H6" s="2">
         <v>6.0</v>
@@ -11897,7 +11909,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16426,22 +16438,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>129</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="H2" s="2">
         <v>7.0</v>
@@ -16452,16 +16464,16 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>752</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>747</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>748</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>743</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>744</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>123</v>
@@ -16475,22 +16487,22 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>208</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>123</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="H4" s="2">
         <v>7.0</v>
@@ -16501,16 +16513,16 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>62</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>123</v>
@@ -16524,16 +16536,16 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>123</v>
@@ -16547,19 +16559,19 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>192</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="H7" s="2">
         <v>7.0</v>
@@ -16570,13 +16582,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>388</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>26</v>
@@ -16585,7 +16597,7 @@
         <v>123</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="H8" s="2">
         <v>7.0</v>
@@ -16596,13 +16608,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>26</v>
@@ -16611,7 +16623,7 @@
         <v>123</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="H9" s="2">
         <v>8.0</v>
@@ -16622,13 +16634,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>62</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>39</v>
@@ -16645,7 +16657,7 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>159</v>
@@ -16668,7 +16680,7 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>208</v>
@@ -16691,10 +16703,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -16714,10 +16726,10 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -16737,10 +16749,10 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -16749,7 +16761,7 @@
         <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="H15" s="2">
         <v>8.0</v>
@@ -16760,10 +16772,10 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -16783,7 +16795,7 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>522</v>
@@ -16806,7 +16818,7 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>75</v>
@@ -16829,7 +16841,7 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>321</v>
@@ -16852,7 +16864,7 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>144</v>
@@ -16875,7 +16887,7 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>125</v>
@@ -16898,7 +16910,7 @@
         <v>21.0</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>263</v>
@@ -16921,7 +16933,7 @@
         <v>22.0</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>167</v>
@@ -16944,7 +16956,7 @@
         <v>23.0</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>94</v>
@@ -16967,10 +16979,10 @@
         <v>24.0</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -16990,7 +17002,7 @@
         <v>25.0</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>79</v>
@@ -17013,7 +17025,7 @@
         <v>26.0</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>20</v>
@@ -17036,7 +17048,7 @@
         <v>27.0</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>267</v>
@@ -17059,7 +17071,7 @@
         <v>28.0</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>51</v>
@@ -17082,7 +17094,7 @@
         <v>29.0</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>180</v>
@@ -17105,10 +17117,10 @@
         <v>30.0</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>10</v>
@@ -17128,7 +17140,7 @@
         <v>31.0</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>90</v>
@@ -17151,7 +17163,7 @@
         <v>32.0</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>175</v>
@@ -17174,7 +17186,7 @@
         <v>33.0</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>177</v>
@@ -17197,7 +17209,7 @@
         <v>34.0</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>516</v>
@@ -17220,10 +17232,10 @@
         <v>35.0</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>10</v>
@@ -17243,7 +17255,7 @@
         <v>36.0</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>165</v>
@@ -17266,10 +17278,10 @@
         <v>37.0</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>10</v>
@@ -17289,7 +17301,7 @@
         <v>38.0</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>20</v>
@@ -17335,7 +17347,7 @@
         <v>40.0</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>25</v>
@@ -17358,10 +17370,10 @@
         <v>41.0</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>10</v>
@@ -17381,10 +17393,10 @@
         <v>42.0</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>10</v>
@@ -17404,7 +17416,7 @@
         <v>43.0</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>148</v>
@@ -17427,10 +17439,10 @@
         <v>44.0</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>10</v>
@@ -17450,10 +17462,10 @@
         <v>45.0</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>10</v>
@@ -17473,7 +17485,7 @@
         <v>46.0</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>477</v>
@@ -17496,10 +17508,10 @@
         <v>47.0</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>10</v>
@@ -17519,7 +17531,7 @@
         <v>48.0</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>300</v>
@@ -17542,7 +17554,7 @@
         <v>49.0</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>278</v>
@@ -17565,10 +17577,10 @@
         <v>50.0</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>10</v>
@@ -17588,7 +17600,7 @@
         <v>51.0</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>271</v>
@@ -17611,10 +17623,10 @@
         <v>52.0</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>10</v>
@@ -17634,10 +17646,10 @@
         <v>53.0</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>10</v>
@@ -17657,10 +17669,10 @@
         <v>54.0</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>10</v>
@@ -17680,7 +17692,7 @@
         <v>55.0</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>90</v>
@@ -17703,10 +17715,10 @@
         <v>56.0</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>10</v>
@@ -17726,7 +17738,7 @@
         <v>57.0</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>192</v>
@@ -17749,7 +17761,7 @@
         <v>58.0</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>15</v>
@@ -17772,10 +17784,10 @@
         <v>59.0</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>10</v>
@@ -17796,10 +17808,10 @@
         <v>60.0</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>10</v>
@@ -17819,7 +17831,7 @@
         <v>61.0</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>403</v>
@@ -17842,7 +17854,7 @@
         <v>62.0</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>377</v>
@@ -17865,7 +17877,7 @@
         <v>63.0</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>532</v>
@@ -17888,10 +17900,10 @@
         <v>64.0</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>10</v>
@@ -17911,7 +17923,7 @@
         <v>65.0</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>144</v>
@@ -17934,7 +17946,7 @@
         <v>66.0</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>15</v>
@@ -17957,7 +17969,7 @@
         <v>67.0</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>129</v>
@@ -17980,7 +17992,7 @@
         <v>68.0</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>75</v>
@@ -17992,7 +18004,7 @@
         <v>26</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="H69" s="2">
         <v>8.0</v>
@@ -18003,7 +18015,7 @@
         <v>69.0</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>388</v>
@@ -18026,7 +18038,7 @@
         <v>70.0</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>496</v>
@@ -18049,10 +18061,10 @@
         <v>71.0</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>10</v>
@@ -18072,7 +18084,7 @@
         <v>72.0</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>433</v>
@@ -18095,7 +18107,7 @@
         <v>73.0</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>208</v>
@@ -18118,7 +18130,7 @@
         <v>74.0</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>477</v>
@@ -26685,6 +26697,9 @@
       <c r="F4" s="1" t="s">
         <v>551</v>
       </c>
+      <c r="G4" s="2" t="s">
+        <v>594</v>
+      </c>
       <c r="H4" s="1">
         <v>5.0</v>
       </c>
@@ -26694,7 +26709,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>522</v>
@@ -26706,10 +26721,10 @@
         <v>21</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="H5" s="1">
         <v>5.0</v>
@@ -26720,7 +26735,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>144</v>
@@ -26732,10 +26747,10 @@
         <v>26</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="H6" s="1">
         <v>5.0</v>
@@ -26746,7 +26761,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>392</v>
@@ -26758,10 +26773,10 @@
         <v>16</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="H7" s="2">
         <v>6.0</v>
@@ -26772,10 +26787,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>10</v>
@@ -26795,7 +26810,7 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>267</v>
@@ -26808,6 +26823,9 @@
       </c>
       <c r="F9" s="1" t="s">
         <v>411</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>607</v>
       </c>
       <c r="H9" s="1">
         <v>7.0</v>
@@ -26818,7 +26836,7 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>267</v>
@@ -26841,7 +26859,7 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>62</v>
@@ -26853,10 +26871,10 @@
         <v>16</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="H11" s="1">
         <v>7.0</v>
@@ -26867,7 +26885,7 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>62</v>
@@ -26879,10 +26897,10 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="H12" s="2">
         <v>7.0</v>
@@ -26893,7 +26911,7 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>477</v>
@@ -26905,10 +26923,10 @@
         <v>26</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="H13" s="2">
         <v>6.0</v>
@@ -27956,22 +27974,22 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="H2" s="1">
         <v>4.0</v>
@@ -27982,22 +28000,22 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>79</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="H3" s="1">
         <v>5.0</v>
@@ -28008,19 +28026,22 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>627</v>
+        <v>629</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>630</v>
       </c>
       <c r="H4" s="1">
         <v>5.0</v>
@@ -28031,10 +28052,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>10</v>
@@ -28054,7 +28075,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>263</v>
@@ -28066,10 +28087,10 @@
         <v>11</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="H6" s="1">
         <v>7.0</v>
@@ -28080,7 +28101,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>437</v>
@@ -28092,10 +28113,10 @@
         <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="H7" s="2">
         <v>6.0</v>
@@ -28106,19 +28127,25 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>639</v>
+        <v>642</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="H8" s="2">
+        <v>6.0</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1"/>
@@ -29169,10 +29196,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>10</v>
@@ -29181,10 +29208,10 @@
         <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="H2" s="1">
         <v>6.0</v>
@@ -29195,10 +29222,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>10</v>
@@ -29207,10 +29234,10 @@
         <v>501</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="H3" s="1">
         <v>6.0</v>
@@ -29221,7 +29248,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>183</v>
@@ -29233,7 +29260,7 @@
         <v>39</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H4" s="2">
         <v>8.0</v>
@@ -29244,22 +29271,22 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H5" s="2">
         <v>6.0</v>
@@ -29270,22 +29297,22 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>129</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="H6" s="2">
         <v>7.0</v>
@@ -29296,7 +29323,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>58</v>
@@ -29308,10 +29335,10 @@
         <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="H7" s="2">
         <v>7.0</v>

</xml_diff>